<commit_message>
carga ob det agosto lista para correr
</commit_message>
<xml_diff>
--- a/data/Taller_DET_Agosto/Carga_ob/elmo_data.xlsx
+++ b/data/Taller_DET_Agosto/Carga_ob/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Taller_DET_Agosto\Carga_ob\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A7E634C-A78F-4B3B-A416-9984B201631C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C55ED14-FAE4-40DE-9C1F-5BF49C892AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -2401,7 +2401,7 @@
         <v>5733</v>
       </c>
       <c r="F3" s="14">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G3" s="8">
         <v>1</v>

</xml_diff>